<commit_message>
Enhance insurance in hospital template, add custom option dropdown, match hero button sizes, show insurance first and adjust mobile search order
</commit_message>
<xml_diff>
--- a/Template - HOSPTIAL Data.xlsx
+++ b/Template - HOSPTIAL Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11114"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ismail/Desktop/00 ISMAIL 2025/  ISAM TRADE LINKS/10 MeetAdr/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Public\meetadr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8C3BFD5-DF6E-BA40-8D9D-94B585D15992}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3F9DCCE-3F16-4FF3-92A5-67613E63C0DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1880" yWindow="2240" windowWidth="26840" windowHeight="15700" xr2:uid="{9BC4E85C-3679-D946-99CE-94A095CE042B}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{9BC4E85C-3679-D946-99CE-94A095CE042B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="31">
   <si>
     <t>Country</t>
   </si>
@@ -124,6 +124,9 @@
   </si>
   <si>
     <t>User_Name</t>
+  </si>
+  <si>
+    <t>Insurance</t>
   </si>
 </sst>
 </file>
@@ -167,7 +170,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -190,19 +193,29 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -517,14 +530,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4E73CB8-8A95-794E-90DC-0E6F4B02208A}">
-  <dimension ref="B1:C20"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="B1:C21"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="33.83203125" customWidth="1"/>
     <col min="3" max="3" width="20.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B1" s="1" t="s">
         <v>15</v>
       </c>
@@ -532,7 +545,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B2" s="2" t="s">
         <v>19</v>
       </c>
@@ -540,7 +553,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B3" s="2" t="s">
         <v>0</v>
       </c>
@@ -548,7 +561,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B4" s="2" t="s">
         <v>5</v>
       </c>
@@ -556,7 +569,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B5" s="2" t="s">
         <v>1</v>
       </c>
@@ -564,7 +577,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B6" s="2" t="s">
         <v>20</v>
       </c>
@@ -572,7 +585,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B7" s="2" t="s">
         <v>2</v>
       </c>
@@ -580,7 +593,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B8" s="2" t="s">
         <v>3</v>
       </c>
@@ -588,7 +601,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B9" s="2" t="s">
         <v>21</v>
       </c>
@@ -596,7 +609,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B10" s="2" t="s">
         <v>22</v>
       </c>
@@ -604,65 +617,73 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B11" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C11" s="3"/>
     </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B12" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C12" s="3"/>
     </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B13" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C13" s="3"/>
     </row>
-    <row r="14" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B14" s="2" t="s">
         <v>25</v>
       </c>
       <c r="C14" s="3"/>
     </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B15" s="6" t="s">
+    <row r="15" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B15" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C15" s="3"/>
     </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B16" s="6" t="s">
+    <row r="16" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B16" s="4" t="s">
         <v>26</v>
       </c>
       <c r="C16" s="3"/>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B17" s="6" t="s">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B17" s="4" t="s">
         <v>27</v>
       </c>
       <c r="C17" s="3"/>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B18" s="6" t="s">
+    <row r="18" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B18" s="4" t="s">
         <v>28</v>
       </c>
       <c r="C18" s="3"/>
     </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B19" s="7" t="s">
+    <row r="19" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B19" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C19" s="6"/>
-    </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B20" s="7" t="s">
+      <c r="C19" s="4"/>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B20" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C20" s="6"/>
+      <c r="C20" s="4"/>
+    </row>
+    <row r="21" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B21" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>17</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>